<commit_message>
Actualización automática 2026-06-15 08:30:19
</commit_message>
<xml_diff>
--- a/data/NOLE MOROCHO MARCIA DEL PILAR.xlsx
+++ b/data/NOLE MOROCHO MARCIA DEL PILAR.xlsx
@@ -647,11 +647,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
@@ -823,144 +823,84 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>TAPIA GONZALES ERIKA MABEL</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="Q4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
-        </is>
-      </c>
-      <c r="R4" s="4" t="inlineStr">
-        <is>
-          <t>0 de 2</t>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>0 de 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-07-03 11:30:17
</commit_message>
<xml_diff>
--- a/data/NOLE MOROCHO MARCIA DEL PILAR.xlsx
+++ b/data/NOLE MOROCHO MARCIA DEL PILAR.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -546,7 +546,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>COQUE TONATO RICHARD PAUL</t>
+          <t>TAPIA GONZALES ERIKA MABEL</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -573,7 +573,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TAPIA GONZALES ERIKA MABEL</t>
+          <t>YANEZ OÑA RICHARD ALEXANDER</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -593,46 +593,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>NOLE MOROCHO MARCIA DEL PILAR</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>YANEZ OÑA RICHARD ALEXANDER</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="C7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="3" t="n">
+      <c r="C6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>